<commit_message>
Phase 4 abgeschlossen: Neue Teamverwaltung mit AssignmentWidget
</commit_message>
<xml_diff>
--- a/Excel/Terminefussball_2026_Herbst.xlsx
+++ b/Excel/Terminefussball_2026_Herbst.xlsx
@@ -5776,7 +5776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.5546875" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -5878,6 +5878,23 @@
         </is>
       </c>
       <c r="E5" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MEMBER000014</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TRAINER</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>JA</t>
         </is>
@@ -5894,7 +5911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="11.77734375" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -6071,7 +6088,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>JA</t>
+          <t>NEIN</t>
         </is>
       </c>
     </row>
@@ -6093,7 +6110,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>JA</t>
+          <t>NEIN</t>
         </is>
       </c>
     </row>
@@ -6115,7 +6132,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>JA</t>
+          <t>NEIN</t>
         </is>
       </c>
     </row>
@@ -6137,7 +6154,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>JA</t>
+          <t>NEIN</t>
         </is>
       </c>
     </row>
@@ -6158,6 +6175,358 @@
         </is>
       </c>
       <c r="F11" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MEMBER000002</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MEMBER000004</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MEMBER000007</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MEMBER000009</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MEMBER000011</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>MEMBER000005</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MEMBER000008</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TEAM000002</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MEMBER000014</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Trainer</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MEMBER000002</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MEMBER000004</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>MEMBER000005</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>MEMBER000007</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MEMBER000008</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>MEMBER000009</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>MEMBER000011</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>MEMBER000012</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TRAINER</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
         <is>
           <t>JA</t>
         </is>
@@ -6174,7 +6543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="17.77734375" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -7647,6 +8016,132 @@
         </is>
       </c>
       <c r="I36" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>02.07.2026 17:09:47</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Mannschaft</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>U16</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Daten aktualisiert</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>gfhfh</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>02.07.2026 17:31:51</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>TEAM000002</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Mannschaft</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Daten aktualisiert</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>02.07.2026 17:54:45</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Mannschaft</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>U16</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Daten aktualisiert</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>sdfsdfgfg</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
         <is>
           <t>System</t>
         </is>
@@ -7752,7 +8247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.5546875" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -8211,6 +8706,38 @@
         </is>
       </c>
       <c r="G14" t="inlineStr">
+        <is>
+          <t>Aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MEMBER000014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Frans</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Posposil</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>01.01.1980</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>02.07.2026</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>Aktiv</t>
         </is>

</xml_diff>

<commit_message>
Phase 5: Trainingsverwaltung mit Teilnehmerstruktur
</commit_message>
<xml_diff>
--- a/Excel/Terminefussball_2026_Herbst.xlsx
+++ b/Excel/Terminefussball_2026_Herbst.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="7" activeTab="12" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="10" activeTab="13" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="ICS2" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,6 +19,8 @@
     <sheet name="CFG_LOOKUPS" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="MEMBER_ROLES" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="TEAM_ASSIGNMENTS" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="TRAININGS" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="TRAINING_PARTICIPANTS" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -6537,13 +6539,313 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TRAINING_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TEAM_ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>DATUM</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>STARTZEIT</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ENDZEIT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ORT</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>TRAINING_TYPE</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>AKTIV</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>BEMERKUNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TRN000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Steinbrunn</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Geplant</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>U11</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Neufeld</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Geplant</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TRN000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>U12</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Steinbrunn</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Geplant</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TRN000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>U13</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Neufeld</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Geplant</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TRAINING_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>MEMBER_ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ROLE</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>BEMERKUNG</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>AKTIV</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="17.77734375" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -8142,6 +8444,171 @@
         </is>
       </c>
       <c r="I39" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>03.07.2026 17:12:57</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>TRN000001</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>03.07.2026 17:24:31</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TRN000001</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Archiviert</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TRN000001</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Training wurde archiviert</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>03.07.2026 17:27:03</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>03.07.2026 17:27:16</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TRN000003</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>03.07.2026 19:14:38</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
         <is>
           <t>System</t>
         </is>

</xml_diff>

<commit_message>
Sprint 10.2.0 - Architektur Fußballmanager vorbereitet
</commit_message>
<xml_diff>
--- a/Excel/Terminefussball_2026_Herbst.xlsx
+++ b/Excel/Terminefussball_2026_Herbst.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="10" activeTab="13" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="11" activeTab="15" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="ICS2" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,6 +21,12 @@
     <sheet name="TEAM_ASSIGNMENTS" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="TRAININGS" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="TRAINING_PARTICIPANTS" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="TRAINING_SCHEDULES" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="CLUB" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="SEASONS" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="FACILITIES" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="PLACES" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="DEPARTMENTS" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -6545,7 +6551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -6783,6 +6789,100 @@
         </is>
       </c>
       <c r="I5" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TRN000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>U16</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>05.07.2026</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Wimpassing</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Geplant</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TRN000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>U7</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>12.07.2026</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Neufeld</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Geplant</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
@@ -6799,38 +6899,677 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TRAINING_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>MEMBER_ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ROLE</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>BEMERKUNG</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>AKTIV</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MEMBER000004</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MEMBER000007</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MEMBER000004</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MEMBER000007</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MEMBER000002</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TRN000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MEMBER000002</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TRN000006</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MEMBER000007</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TRN000006</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MEMBER000011</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TRN000006</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MEMBER000014</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TRAINER</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MEMBER000004</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MEMBER000007</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MEMBER000002</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TRAINER</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MEMBER000002</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TRAINER</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MEMBER000004</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CO_TRAINER</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MEMBER000007</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>TRN000004</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>MEMBER000012</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CO_TRAINER</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TRN000004</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MEMBER000004</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TRN000004</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MEMBER000010</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TRN000004</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MEMBER000007</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TRAINER</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TRN000004</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MEMBER000013</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TRAINER</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>SCHEDULE_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TEAM_ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>SAISON</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>WOCHENTAG</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>BEGINN</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ENDE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>PLATZ</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>TRAINING_TYPE</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>AKTIV</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>BEMERKUNG</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CLUB_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>LANDESVERBAND</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>LOGO</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>AKTIV</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>TRAINING_ID</t>
+          <t>SAISON_ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>MEMBER_ID</t>
+          <t>NAME</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>ROLE</t>
+          <t>VON</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>STATUS</t>
+          <t>BIS</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>AKTIV</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>BEMERKUNG</t>
         </is>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>FACILITY_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ORT</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ADRESSE</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>AKTIV</t>
+        </is>
+      </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>AKTIV</t>
+          <t>BEMERKUNG</t>
         </is>
       </c>
     </row>
@@ -6845,7 +7584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="17.77734375" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -8611,6 +9350,295 @@
       <c r="I44" t="inlineStr">
         <is>
           <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>04.07.2026 10:54:40</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>04.07.2026 11:47:23</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>04.07.2026 20:36:19</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>TRN000006</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>12.07.2026</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>05.07.2026 09:59:24</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>05.07.2026 11:37:23</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>TRN000002</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>05.07.2026 12:35:55</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>TRN000004</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>03.07.2026</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>PLACE_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>FACILITY_ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>TRAINING_KAPAZITAET</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>IST_SPIELPLATZ</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>SPIEL_KAPAZITAET</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>AKTIV</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>BEMERKUNG</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>DEPARTMENT_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>LEITER_MEMBER_ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>AKTIV</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>BEMERKUNG</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 10.5.0 - Erstes Verwaltungsmodul abgeschlossen
</commit_message>
<xml_diff>
--- a/Excel/Terminefussball_2026_Herbst.xlsx
+++ b/Excel/Terminefussball_2026_Herbst.xlsx
@@ -9612,7 +9612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9639,6 +9639,91 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>BEMERKUNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DEP000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Nachwuchs</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DEP000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Futsall</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DEP000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TEst5</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DEP000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DEP000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Test2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Nein</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 47 - Trainingsmanagement inkl. WarningDialog und Kollisionsprüfung
</commit_message>
<xml_diff>
--- a/Excel/Terminefussball_2026_Herbst.xlsx
+++ b/Excel/Terminefussball_2026_Herbst.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="14" activeTab="17" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="14" activeTab="20" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="ICS2" sheetId="1" state="visible" r:id="rId1"/>
@@ -5759,7 +5759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.5546875" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -6066,7 +6066,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>JA</t>
+          <t>NEIN</t>
         </is>
       </c>
     </row>
@@ -6099,6 +6099,23 @@
         </is>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MEMBER000013</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>JA</t>
         </is>
@@ -7801,8 +7818,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="12.44140625" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
+    <col width="11.77734375" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
+    <col width="9.77734375" bestFit="1" customWidth="1" style="4" min="3" max="3"/>
+    <col width="12.109375" bestFit="1" customWidth="1" style="4" min="4" max="4"/>
+    <col width="7.5546875" bestFit="1" customWidth="1" style="4" min="5" max="5"/>
+    <col width="5.5546875" bestFit="1" customWidth="1" style="4" min="6" max="6"/>
+    <col width="10" bestFit="1" customWidth="1" style="4" min="7" max="7"/>
+    <col width="5.5546875" bestFit="1" customWidth="1" style="4" min="8" max="8"/>
+    <col width="14.21875" bestFit="1" customWidth="1" style="4" min="9" max="9"/>
+    <col width="5.77734375" bestFit="1" customWidth="1" style="4" min="10" max="10"/>
+    <col width="11.77734375" bestFit="1" customWidth="1" style="4" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -7837,22 +7867,359 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>PLATZ</t>
+          <t>PLACE_ID</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>ZONE</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>TRAINING_TYPE</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>AKTIV</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>BEMERKUNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SCH000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Montag</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PLA000004</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Test Bearbeiten</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SCH000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TEAM000002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Montag</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PLA000004</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Test1234</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SCH000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TEAM000002</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Montag</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PLA000005</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>test1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SCH000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TEAM000003</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Mittwoch</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PLA000004</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>u7test</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SCH000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Montag</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PLA000005</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SCH000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TEAM000004</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Montag</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PLA000005</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Ja</t>
         </is>
       </c>
     </row>
@@ -8012,7 +8379,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Futsall</t>
+          <t>KM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -8034,7 +8401,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nein</t>
         </is>
       </c>
     </row>
@@ -8197,7 +8564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="17.77734375" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -10827,6 +11194,265 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>13.07.2026 22:29:08</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>TEAM000001</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Mannschaft</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Tippfehler korrigiert</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>14.07.2026 07:01:00</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>TEAM000001</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Mannschaft</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Daten aktualisiert</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>14.07.2026 09:32:14</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>TEAM000001</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Mannschaft</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Vereinsentscheidung</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>14.07.2026 10:13:38</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>TEAM000001</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Mannschaft</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Tippfehler korrigiert</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>14.07.2026 11:51:13</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>TEAM000002</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Mannschaft</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Tippfehler korrigiert</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>14.07.2026 12:16:06</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>TEAM000001</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Mannschaft</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Tippfehler korrigiert</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>14.07.2026 13:12:12</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>MEMBER000013</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Mitglied</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Bearbeitet</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Dieter Berger</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Tippfehler korrigiert</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10838,7 +11464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.88671875" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
@@ -10903,6 +11529,11 @@
           <t>BEMERKUNG</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>TRAININGSZONEN</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -10944,8 +11575,11 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Ja</t>
-        </is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -10966,8 +11600,58 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PLA000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>FAC000003</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Trainingsplatz</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>Ja</t>
         </is>
+      </c>
+      <c r="K5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PLA000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>FAC000002</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hauptplatz</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -10984,7 +11668,7 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="8.5546875" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
+    <col width="11.77734375" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
     <col width="6.109375" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
     <col width="12.77734375" bestFit="1" customWidth="1" style="4" min="3" max="3"/>
     <col width="15.21875" bestFit="1" customWidth="1" style="4" min="4" max="4"/>
@@ -11042,7 +11726,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DEP000001</t>
+          <t>DEP000002</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -11069,7 +11753,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DEP000001</t>
+          <t>DEP000002</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -11134,6 +11818,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
@@ -11143,18 +11828,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="17.21875" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
-    <col width="8.5546875" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
-    <col width="11.33203125" bestFit="1" customWidth="1" style="4" min="3" max="3"/>
-    <col width="6.21875" bestFit="1" customWidth="1" style="4" min="4" max="4"/>
-    <col width="4.77734375" bestFit="1" customWidth="1" style="4" min="5" max="5"/>
-    <col width="3.5546875" bestFit="1" customWidth="1" style="4" min="6" max="6"/>
-    <col width="5.77734375" bestFit="1" customWidth="1" style="4" min="7" max="7"/>
-    <col width="11.77734375" bestFit="1" customWidth="1" style="4" min="8" max="8"/>
-  </cols>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -11195,6 +11870,222 @@
       <c r="H1" t="inlineStr">
         <is>
           <t>BEMERKUNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TM000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TEAM000001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MEMBER000013</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TM000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TEAM000001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MEMBER000002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TM000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TEAM000002</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MEMBER000013</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TM000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TEAM000002</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MEMBER000002</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TM000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TEAM000001</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MEMBER000012</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TM000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TEAM000003</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MEMBER000002</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SPIELER</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TM000007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TEAM000002</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MEMBER000002</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TRAINER</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TM000008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TEAM000002</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MEMBER000014</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>TRAINER</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Ja</t>
         </is>
       </c>
     </row>
@@ -11810,12 +12701,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>006487965432</t>
+          <t>6456487965432.0</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>123456</t>
+          <t>123456.0</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">

</xml_diff>